<commit_message>
DTP lists: About sheet and provenance carry the modal's corrections
</commit_message>
<xml_diff>
--- a/public/downloads/suffolk-dtp-lists.xlsx
+++ b/public/downloads/suffolk-dtp-lists.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -431,7 +431,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Suffolk County DA decline-to-prosecute classification</t>
+          <t>Decline-to-prosecute classification worksheet, made inside the Suffolk County District Attorney's office, 2020</t>
         </is>
       </c>
     </row>
@@ -441,7 +441,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>This workbook lists every charge description in the Suffolk County District Attorney's office's decline-to-prosecute classification: which of four categories, decline (YY), presumption against (NY), case-by-case (NS), or ordinarily prosecuted (NN), the office's worksheet assigns to it.</t>
+          <t>This workbook lists every charge description in a decline-to-prosecute classification worksheet made inside the Suffolk County District Attorney's office: which of four categories, decline (YY), presumption against (NY), case-by-case (NS), or ordinarily prosecuted (NN), the worksheet assigns to it.</t>
         </is>
       </c>
     </row>
@@ -462,24 +462,65 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>The Review tier column carries the three sections of the worksheet's 2020 review tab: 'Current list', 'Proposed, agreed (never adopted)', and 'Proposed, disagreed'. A blank Review tier means the review never covered that description.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>This file is derived from that worksheet. The worksheet itself is not distributed. Generated 2026-08-13.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>The decline list (YY) sheet is broader than the operative list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>The worksheet's YY tab holds 69 charge descriptions, and the 'Decline list (YY)' sheet carries all 69. The operative list is the narrower set of 46, the rows marked 'Current list' in the Review tier column. The extras include drug distribution charges the worksheet's own annotations say were not in the memo. The worksheet records no adoption of the expansion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Where the two count columns come from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Both columns come from the assembled charge-level files behind this project's explorer. 'Charges filed 2022-2025' counts charges filed 2022 to 2025 in the 2022-2025 file; 'Charges filed 2006-2021' counts charges filed 2006 to 2021 in the pre-2022 file. Each column counts every charge filed in that window across the whole file, whatever the explorer is filtered to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Conflicts.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Some charge descriptions are marked class YY (on the decline list) while the worksheet's own review tab separately proposed changing that description's category and recorded a reviewer's disagreement. The 'Conflicts' rows in the 'All lists' sheet are these charge descriptions: 10 distinct descriptions, covering 2,393 charges filed 2022 to 2025.</t>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Some charge descriptions are marked class YY (on the decline list) while the worksheet's own review tab separately proposed changing that description's category and recorded a reviewer's disagreement. To find them, take the rows where Class is 'YY (decline list)' and Review tier is 'Proposed, disagreed': 10 distinct descriptions, covering 2,393 charges filed 2022 to 2025.</t>
         </is>
       </c>
     </row>

</xml_diff>